<commit_message>
Compared one day's expired orders with executed orders and then compared the result with previous day's expired orders
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/order_files/Mapped_Expired_OrderBook_Equity_24july2026_Fri.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/order_files/Mapped_Expired_OrderBook_Equity_24july2026_Fri.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\order_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77B72CE3-2F5C-414D-832C-C26F9E3D7D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92191C48-2AE4-45D5-A0CB-495256D16DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$114</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -574,6 +577,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E114"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="18.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -2514,6 +2520,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B1:B114" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>